<commit_message>
added the products,userregister and commonapis are created
</commit_message>
<xml_diff>
--- a/Digital_Village_Api/Data/user.xlsx
+++ b/Digital_Village_Api/Data/user.xlsx
@@ -191,6 +191,27 @@
   </x:si>
   <x:si>
     <x:t>12-08-2026 12:07:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>madhu General store</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6789067890</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13-08-2026 19:20:39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13-08-2026 19:21:42</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1034,6 +1055,136 @@
         <x:v>52</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" spans="1:21">
+      <x:c r="A9" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I9" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J9" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K9" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="L9" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="M9" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="N9" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="O9" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="P9" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="Q9" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="R9" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="S9" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="T9" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="U9" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:21">
+      <x:c r="A10" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H10" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="I10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J10" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="K10" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="L10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="M10" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="N10" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="O10" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="P10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="Q10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="R10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="S10" s="0" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="T10" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="U10" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>